<commit_message>
feat: setup whatsapp official health check
</commit_message>
<xml_diff>
--- a/docs/tracker_tahapan_pengembangan.xlsx.xlsx
+++ b/docs/tracker_tahapan_pengembangan.xlsx.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Zulfano\Zulfano\Binus\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Zulfano\Zulfano\Binus\whatsapp-bot-rekonsiliasi\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B289D98-AE8A-415A-B70C-65BA9874EAC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E139067-D346-4E9D-825E-0EC3E0CB8C0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{50BE75E0-1459-40E2-B31B-6E549EBCEF56}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{50BE75E0-1459-40E2-B31B-6E549EBCEF56}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="163">
   <si>
     <t>No</t>
   </si>
@@ -474,6 +475,87 @@
   </si>
   <si>
     <t>Bab konsisten</t>
+  </si>
+  <si>
+    <t>Commit &amp; push tahap perencanaan</t>
+  </si>
+  <si>
+    <t>Tahap perencanaan terdokumentasi</t>
+  </si>
+  <si>
+    <t>docs: finalize project planning</t>
+  </si>
+  <si>
+    <t>Commit &amp; push tahap database</t>
+  </si>
+  <si>
+    <t>Skema database final</t>
+  </si>
+  <si>
+    <t>Commit &amp; push tahap backend</t>
+  </si>
+  <si>
+    <t>Backend terhubung database</t>
+  </si>
+  <si>
+    <t>feat: setup backend and mysql connection</t>
+  </si>
+  <si>
+    <t>Commit &amp; push tahap WhatsApp layer</t>
+  </si>
+  <si>
+    <t>Integrasi WhatsApp siap</t>
+  </si>
+  <si>
+    <t>feat: setup whatsapp official integration</t>
+  </si>
+  <si>
+    <t>Commit &amp; push tahap bot logic</t>
+  </si>
+  <si>
+    <t>Fitur bot utama selesai</t>
+  </si>
+  <si>
+    <t>feat: implement bot command features</t>
+  </si>
+  <si>
+    <t>Commit &amp; push tahap keamanan</t>
+  </si>
+  <si>
+    <t>Sistem whitelist aktif</t>
+  </si>
+  <si>
+    <t>feat: implement whitelist management</t>
+  </si>
+  <si>
+    <t>Commit &amp; push fitur pendukung</t>
+  </si>
+  <si>
+    <t>File &amp; logging stabil</t>
+  </si>
+  <si>
+    <t>feat: add file handling and logging</t>
+  </si>
+  <si>
+    <t>Commit &amp; push hasil pengujian</t>
+  </si>
+  <si>
+    <t>Hasil uji terdokumentasi</t>
+  </si>
+  <si>
+    <t>Commit &amp; push dokumentasi akhir</t>
+  </si>
+  <si>
+    <t>Dokumentasi final</t>
+  </si>
+  <si>
+    <t>docs: finalize thesis documentation</t>
+  </si>
+  <si>
+    <t>Commit &amp; push final proyek</t>
+  </si>
+  <si>
+    <t>Proyek final</t>
   </si>
 </sst>
 </file>
@@ -502,12 +584,18 @@
       <name val="Arial Unicode MS"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -548,16 +636,18 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
           <xfpb:xfComplement i="0"/>
         </ext>
       </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -913,13 +1003,13 @@
   <dimension ref="A1:G29"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="4.453125" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.90625" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.90625" style="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.08984375" style="5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.08984375" style="5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="34.08984375" style="5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.1796875" style="5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.08984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="34.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -941,77 +1031,77 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="1" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" s="2">
+      <c r="A2" s="5">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="G2" s="6" t="b">
-        <v>0</v>
+      <c r="G2" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" s="2">
+      <c r="A3" s="5">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="6" t="b">
-        <v>0</v>
+      <c r="G3" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:7">
-      <c r="A4" s="2">
+      <c r="A4" s="5">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="6" t="b">
-        <v>0</v>
+      <c r="G4" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -1033,7 +1123,7 @@
       <c r="F5" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="G5" s="6" t="b">
+      <c r="G5" s="4" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1056,7 +1146,7 @@
       <c r="F6" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="G6" s="6" t="b">
+      <c r="G6" s="4" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1079,7 +1169,7 @@
       <c r="F7" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="G7" s="6" t="b">
+      <c r="G7" s="4" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1102,7 +1192,7 @@
       <c r="F8" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="G8" s="6" t="b">
+      <c r="G8" s="4" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1125,7 +1215,7 @@
       <c r="F9" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="G9" s="6" t="b">
+      <c r="G9" s="4" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1148,7 +1238,7 @@
       <c r="F10" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="G10" s="6" t="b">
+      <c r="G10" s="4" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1171,7 +1261,7 @@
       <c r="F11" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="G11" s="6" t="b">
+      <c r="G11" s="4" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1194,7 +1284,7 @@
       <c r="F12" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="G12" s="6" t="b">
+      <c r="G12" s="4" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1217,7 +1307,7 @@
       <c r="F13" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="G13" s="6" t="b">
+      <c r="G13" s="4" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1240,7 +1330,7 @@
       <c r="F14" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="G14" s="6" t="b">
+      <c r="G14" s="4" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1263,7 +1353,7 @@
       <c r="F15" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="G15" s="6" t="b">
+      <c r="G15" s="4" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1286,7 +1376,7 @@
       <c r="F16" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="G16" s="6" t="b">
+      <c r="G16" s="4" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1309,7 +1399,7 @@
       <c r="F17" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="G17" s="6" t="b">
+      <c r="G17" s="4" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1332,7 +1422,7 @@
       <c r="F18" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="G18" s="6" t="b">
+      <c r="G18" s="4" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1355,7 +1445,7 @@
       <c r="F19" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G19" s="6" t="b">
+      <c r="G19" s="4" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1378,7 +1468,7 @@
       <c r="F20" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="G20" s="6" t="b">
+      <c r="G20" s="4" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1401,7 +1491,7 @@
       <c r="F21" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="G21" s="6" t="b">
+      <c r="G21" s="4" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1424,7 +1514,7 @@
       <c r="F22" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="G22" s="6" t="b">
+      <c r="G22" s="4" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1447,7 +1537,7 @@
       <c r="F23" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="G23" s="6" t="b">
+      <c r="G23" s="4" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1470,7 +1560,7 @@
       <c r="F24" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="G24" s="6" t="b">
+      <c r="G24" s="4" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1493,7 +1583,7 @@
       <c r="F25" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="G25" s="6" t="b">
+      <c r="G25" s="4" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1516,7 +1606,7 @@
       <c r="F26" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="G26" s="6" t="b">
+      <c r="G26" s="4" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1539,7 +1629,7 @@
       <c r="F27" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="G27" s="6" t="b">
+      <c r="G27" s="4" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1562,7 +1652,7 @@
       <c r="F28" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="G28" s="6" t="b">
+      <c r="G28" s="4" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1585,7 +1675,845 @@
       <c r="F29" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="G29" s="6" t="b">
+      <c r="G29" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45DB6D8D-6F1D-4F77-94BC-8A80F03CA2DA}">
+  <dimension ref="A1:G38"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="3.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="30.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="34.81640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" s="5">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="5"/>
+      <c r="G2" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" s="5">
+        <v>2</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="5"/>
+      <c r="G3" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="5">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="F4" s="5"/>
+      <c r="G4" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" s="5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="G5" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" s="5">
+        <v>5</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="F6" s="5"/>
+      <c r="G6" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" s="5">
+        <v>6</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="F7" s="5"/>
+      <c r="G7" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" s="5">
+        <v>7</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8" s="5"/>
+      <c r="G8" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" s="5">
+        <v>8</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F9" s="5"/>
+      <c r="G9" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" s="5">
+        <v>9</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="G10" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" s="5">
+        <v>10</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F11" s="5"/>
+      <c r="G11" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" s="5">
+        <v>11</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="F12" s="5"/>
+      <c r="G12" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="24.5" customHeight="1">
+      <c r="A13" s="5">
+        <v>12</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="G13" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" s="5">
+        <v>13</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="F14" s="5"/>
+      <c r="G14" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" s="5">
+        <v>14</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="F15" s="5"/>
+      <c r="G15" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" s="5">
+        <v>15</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="F16" s="5"/>
+      <c r="G16" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" s="2">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="G17" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" s="2">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F18" s="2"/>
+      <c r="G18" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" s="2">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="F19" s="2"/>
+      <c r="G19" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20" s="2">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F20" s="2"/>
+      <c r="G20" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" s="2">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="F21" s="2"/>
+      <c r="G21" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" s="2">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="G22" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" s="2">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F23" s="2"/>
+      <c r="G23" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24" s="2">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F24" s="2"/>
+      <c r="G24" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="A25" s="2">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="F25" s="2"/>
+      <c r="G25" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="A26" s="2">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="G26" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7">
+      <c r="A27" s="2">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="F27" s="2"/>
+      <c r="G27" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
+      <c r="A28" s="2">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="F28" s="2"/>
+      <c r="G28" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29" s="2">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="F29" s="2"/>
+      <c r="G29" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7">
+      <c r="A30" s="2">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="F30" s="2"/>
+      <c r="G30" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7">
+      <c r="A31" s="2">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="G31" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7">
+      <c r="A32" s="2">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="F32" s="2"/>
+      <c r="G32" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7">
+      <c r="A33" s="2">
+        <v>32</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F33" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="G33" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7">
+      <c r="A34" s="2">
+        <v>33</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="F34" s="2"/>
+      <c r="G34" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7">
+      <c r="A35" s="2">
+        <v>34</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F35" s="2"/>
+      <c r="G35" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7">
+      <c r="A36" s="2">
+        <v>35</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="G36" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7">
+      <c r="A37" s="2">
+        <v>36</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="F37" s="2"/>
+      <c r="G37" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7">
+      <c r="A38" s="2">
+        <v>37</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F38" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="G38" s="4" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implement prefix askbot and cek command with excel export
</commit_message>
<xml_diff>
--- a/docs/tracker_tahapan_pengembangan.xlsx.xlsx
+++ b/docs/tracker_tahapan_pengembangan.xlsx.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Zulfano\Zulfano\Binus\whatsapp-bot-rekonsiliasi\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E139067-D346-4E9D-825E-0EC3E0CB8C0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65B54071-F627-47BB-9763-6D325606C691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{50BE75E0-1459-40E2-B31B-6E549EBCEF56}"/>
   </bookViews>
@@ -2017,7 +2017,7 @@
       </c>
       <c r="F15" s="5"/>
       <c r="G15" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -2038,93 +2038,93 @@
       </c>
       <c r="F16" s="5"/>
       <c r="G16" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:7">
-      <c r="A17" s="2">
+      <c r="A17" s="5">
         <v>16</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C17" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="D17" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="E17" s="2" t="s">
+      <c r="E17" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="F17" s="3" t="s">
+      <c r="F17" s="6" t="s">
         <v>146</v>
       </c>
       <c r="G17" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:7">
-      <c r="A18" s="2">
+      <c r="A18" s="5">
         <v>17</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="C18" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="D18" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="E18" s="2" t="s">
+      <c r="E18" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="F18" s="2"/>
+      <c r="F18" s="5"/>
       <c r="G18" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:7">
-      <c r="A19" s="2">
+      <c r="A19" s="5">
         <v>18</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="C19" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="D19" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="E19" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="F19" s="2"/>
+      <c r="F19" s="5"/>
       <c r="G19" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:7">
-      <c r="A20" s="2">
+      <c r="A20" s="5">
         <v>19</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C20" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="D20" s="2" t="s">
+      <c r="D20" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="E20" s="2" t="s">
+      <c r="E20" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="F20" s="2"/>
+      <c r="F20" s="5"/>
       <c r="G20" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:7">

</xml_diff>

<commit_message>
feat: add error handling for webhook and excel processing
</commit_message>
<xml_diff>
--- a/docs/tracker_tahapan_pengembangan.xlsx.xlsx
+++ b/docs/tracker_tahapan_pengembangan.xlsx.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Zulfano\Zulfano\Binus\whatsapp-bot-rekonsiliasi\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65B54071-F627-47BB-9763-6D325606C691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23789064-99AE-43E4-AE52-F29DB4860555}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{50BE75E0-1459-40E2-B31B-6E549EBCEF56}"/>
   </bookViews>
@@ -2128,133 +2128,133 @@
       </c>
     </row>
     <row r="21" spans="1:7">
-      <c r="A21" s="2">
+      <c r="A21" s="5">
         <v>20</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C21" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="D21" s="2" t="s">
+      <c r="D21" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="E21" s="2" t="s">
+      <c r="E21" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="F21" s="2"/>
+      <c r="F21" s="5"/>
       <c r="G21" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:7">
-      <c r="A22" s="2">
+      <c r="A22" s="5">
         <v>21</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C22" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="D22" s="2" t="s">
+      <c r="D22" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="E22" s="2" t="s">
+      <c r="E22" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="F22" s="3" t="s">
+      <c r="F22" s="6" t="s">
         <v>149</v>
       </c>
       <c r="G22" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:7">
-      <c r="A23" s="2">
+      <c r="A23" s="5">
         <v>22</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B23" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="C23" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="D23" s="2" t="s">
+      <c r="D23" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="E23" s="2" t="s">
+      <c r="E23" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="F23" s="2"/>
+      <c r="F23" s="5"/>
       <c r="G23" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:7">
-      <c r="A24" s="2">
+      <c r="A24" s="5">
         <v>23</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C24" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="D24" s="2" t="s">
+      <c r="D24" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="E24" s="2" t="s">
+      <c r="E24" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="F24" s="2"/>
+      <c r="F24" s="5"/>
       <c r="G24" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:7">
-      <c r="A25" s="2">
+      <c r="A25" s="5">
         <v>24</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B25" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="C25" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="D25" s="2" t="s">
+      <c r="D25" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="E25" s="2" t="s">
+      <c r="E25" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="F25" s="2"/>
+      <c r="F25" s="5"/>
       <c r="G25" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:7">
-      <c r="A26" s="2">
+      <c r="A26" s="5">
         <v>25</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="C26" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="D26" s="2" t="s">
+      <c r="D26" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="E26" s="2" t="s">
+      <c r="E26" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="F26" s="3" t="s">
+      <c r="F26" s="6" t="s">
         <v>152</v>
       </c>
       <c r="G26" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:7">

</xml_diff>